<commit_message>
ORR v2: Dan is owner and maintainer of Precharge Pro and the reporting tools; the sessions build them
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:K39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col width="2.5703125" customWidth="1" style="14" min="1" max="1"/>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Reporting-tools maintainer session</t>
+          <t>Dan Plant (built with the reporting-tools session)</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>Via Dan Plant. Changes announced before they ship.</t>
+          <t>Dan Plant. Changes announced in the rolling handoff before they ship.</t>
         </is>
       </c>
     </row>
@@ -2833,17 +2833,17 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Precharge Pro maintainer session</t>
+          <t>Dan Plant (built with the Precharge Pro session)</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Dan Plant (precharge responsible)</t>
+          <t>Dan Plant</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Dan Plant</t>
+          <t>Lee Arnold</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="F11" s="19" t="inlineStr">
         <is>
-          <t>Via Dan Plant. MOC register.</t>
+          <t>Dan Plant. MOC register (Synergi #1856051). Sole authority for the precharge password.</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer via Dan</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer via Dan</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer via Dan</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer via Dan</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer via Dan</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer via Dan</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer via Dan</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="F4" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4356,7 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="F18" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="F19" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="F21" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="F23" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="F24" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="F25" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4676,7 +4676,7 @@
       </c>
       <c r="F26" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer / Dan</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer / Dan</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4740,7 +4740,7 @@
       </c>
       <c r="F28" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4772,7 @@
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
       </c>
       <c r="F30" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
     </row>
@@ -6142,7 +6142,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Reporting-tools, Precharge Pro, COC tracker and SPARC maintainers, via Dan</t>
+          <t>Dan Plant (reporting tools and Precharge Pro, with their build sessions); Lee's maintainers for COC tracker and SPARC</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>Precharge maintainer via Dan</t>
+          <t>Dan Plant (Precharge Pro owner and maintainer)</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
@@ -6292,7 +6292,7 @@
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>Tools maintainer via Dan</t>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Lee's tool maintainers via Lee</t>
+          <t>Lee Arnold's tool maintainers</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Programme chart draft 4: transfer in the week of 19 October; production home (sandbox server) as critical item M2a
ORR workbook v2 and gap report v2.1 carry the transfer week and the new Open actions row; IT email and Teams message updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -842,7 +842,7 @@
     <row r="5" ht="11.25" customFormat="1" customHeight="1" s="7">
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>Live version 2, 30 September 2026 (v1 plus the reporting-tools and Precharge Pro maintainers' returns; COC tracker and SPARC still to come via Lee) · prepared by Dan Plant (service owner) · server handover Sunday 18 October 2026 with Adam Snyder</t>
+          <t>Live version 2, 30 September 2026 (v1 plus the reporting-tools and Precharge Pro maintainers' returns; COC tracker and SPARC still to come via Lee) · prepared by Dan Plant (service owner) · server handover Sunday week of 19 October 2026 with Adam Snyder</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
       <c r="I10" s="19" t="inlineStr"/>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>Dan Plant, Technical Superintendent WCE, owns the service (script, dashboards, flows, agent). Lee Arnold, WCE Manager, is co-owner on the agent and the flows and holds the cost centre. ISIT own the server scheduled task from 18 October (Adam Snyder).</t>
+          <t>Dan Plant, Technical Superintendent WCE, owns the service (script, dashboards, flows, agent). Lee Arnold, WCE Manager, is co-owner on the agent and the flows and holds the cost centre. ISIT own the server scheduled task from week of 19 October (Adam Snyder).</t>
         </is>
       </c>
       <c r="K10" s="21" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>RACI drafted on the "Support Model (RACI)" sheet of this workbook. ISIT to confirm their column by 18 Oct. Owner: Dan and ISIT PMO.</t>
+          <t>RACI drafted on the "Support Model (RACI)" sheet of this workbook. ISIT to confirm their column by week of 19 Oct. Owner: Dan and ISIT PMO.</t>
         </is>
       </c>
     </row>
@@ -1161,12 +1161,12 @@
       </c>
       <c r="J14" s="19" t="inlineStr">
         <is>
-          <t>Proposed early-life support: 18 Oct to 6 Nov the scanner runs on the server and on Dan's PC in parallel (dual run, two clean weeks), Dan on call; 6 Nov to Feb 2027 ISIT shadow-run the task with Dan supporting the script until ISIT accept it as a supported service (M11). Not yet reviewed with ISIT.</t>
+          <t>Proposed early-life support: week of 19 Oct to 13 Nov the scanner runs on the server and on Dan's PC in parallel (dual run, two clean weeks), Dan on call; 6 Nov to Feb 2027 ISIT shadow-run the task with Dan supporting the script until ISIT accept it as a supported service (M11). Not yet reviewed with ISIT.</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>Programme chart M5, M7, M11; "DR and early-life support" sheet. Owner: Dan to propose, ISIT PM to accept. Date: 18 Oct.</t>
+          <t>Programme chart M5, M7, M11; "DR and early-life support" sheet. Owner: Dan to propose, ISIT PM to accept. Date: week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
-          <t>HANDOFF.md; SCANNER-SERVER-MIGRATION-IT-HANDOFF.md §3 to §7; *-INSTALL-GUIDE.md; *-FLOW-GUIDE.md; scripts/Archive-ProblemFiles.ps1. Owner: ISIT to review after the 18 Oct transfer. Date: 6 Nov. tools/received/orr/ORR-Reporting-Tools/01-Runbook-ORR-6-7.md; ORR-RETURN-PRECHARGE-PRO.md §1.</t>
+          <t>HANDOFF.md; SCANNER-SERVER-MIGRATION-IT-HANDOFF.md §3 to §7; *-INSTALL-GUIDE.md; *-FLOW-GUIDE.md; scripts/Archive-ProblemFiles.ps1. Owner: ISIT to review after the week of 19 Oct transfer. Date: 6 Nov. tools/received/orr/ORR-Reporting-Tools/01-Runbook-ORR-6-7.md; ORR-RETURN-PRECHARGE-PRO.md §1.</t>
         </is>
       </c>
     </row>
@@ -1263,12 +1263,12 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>Documentation is current to scanner v2.74 (30 Sep) and every change is recorded before it ships. Not yet updated for the server: the server config (paths, service account, notifications off) is written on 18 Oct. Backups: SharePoint is the system of record and the share is regenerated from it by the scanner; the scanner state files on D:\TSC-Dashboard need a server backup (ISIT). Monitoring: see 13.</t>
+          <t>Documentation is current to scanner v2.74 (30 Sep) and every change is recorded before it ships. Not yet updated for the server: the server config (paths, service account, notifications off) is written on week of 19 Oct. Backups: SharePoint is the system of record and the share is regenerated from it by the scanner; the scanner state files on D:\TSC-Dashboard need a server backup (ISIT). Monitoring: see 13.</t>
         </is>
       </c>
       <c r="K16" s="21" t="inlineStr">
         <is>
-          <t>HANDOFF.md (v2.44 to v2.74); config.server.json to be written 18 Oct. Owner: Dan (docs), ISIT (backup of D:\TSC-Dashboard). Date: 18 Oct.</t>
+          <t>HANDOFF.md (v2.44 to v2.74); config.server.json to be written week of 19 Oct. Owner: Dan (docs), ISIT (backup of D:\TSC-Dashboard). Date: week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1314,12 @@
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t>Users need only a browser (PC, iPad, phone); nothing is installed. The server needs Windows PowerShell 5.1 (present) and a way for the three SharePoint report libraries to reach it. Today that is OneDrive sync under Dan's account; under a service account on a server the choice is still open (migration handoff §2: scheduled SharePoint pull recommended, or sync under the service account). This is the one thing that stops the server scanner reading anything and must be decided before 18 Oct.</t>
+          <t>Users need only a browser (PC, iPad, phone); nothing is installed. The server needs Windows PowerShell 5.1 (present) and a way for the three SharePoint report libraries to reach it. Today that is OneDrive sync under Dan's account; under a service account on a server the choice is still open (migration handoff §2: scheduled SharePoint pull recommended, or sync under the service account). This is the one thing that stops the server scanner reading anything and must be decided before week of 19 Oct.</t>
         </is>
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
-          <t>SCANNER-SERVER-MIGRATION-IT-HANDOFF.md §2 (options A and B). Owner: Adam Snyder / ISIT with Dan. Date: decision by 10 Oct, built 18 Oct.</t>
+          <t>SCANNER-SERVER-MIGRATION-IT-HANDOFF.md §2 (options A and B). Owner: Adam Snyder / ISIT with Dan. Date: decision by 10 Oct, built week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1510,7 @@
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="19" t="inlineStr">
         <is>
-          <t>The scanner runs as a scheduled task every ten minutes (Dan's PC today, server from 18 Oct). Notifications are event-driven flows on the post. The Maximo item export runs daily at 06:00 Houston (Manpreet). The AAB overdue chase runs daily from a scanner-written file. Backups are ISIT's (see 7). The hourly Digests freshness alert flow is scheduled to be built by 9 Oct.</t>
+          <t>The scanner runs as a scheduled task every ten minutes (Dan's PC today, server from week of 19 Oct). Notifications are event-driven flows on the post. The Maximo item export runs daily at 06:00 Houston (Manpreet). The AAB overdue chase runs daily from a scanner-written file. Backups are ISIT's (see 7). The hourly Digests freshness alert flow is scheduled to be built by 9 Oct.</t>
         </is>
       </c>
       <c r="K21" s="21" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="J22" s="19" t="inlineStr">
         <is>
-          <t>In place: the dashboard header shows "Data updated N minutes ago" with amber banners when stale; every scan writes a log and a last-successful-scan stamp; Power Automate emails the flow owner on any failed run; Copilot Studio analytics for the agent. Missing: the hourly check that emails Dan and Lee when no digest has been written for two hours (promised to IT, build by 9 Oct), and ISIT task monitoring on the server after 18 Oct. No metrics dashboard in ISIT tooling.</t>
+          <t>In place: the dashboard header shows "Data updated N minutes ago" with amber banners when stale; every scan writes a log and a last-successful-scan stamp; Power Automate emails the flow owner on any failed run; Copilot Studio analytics for the agent. Missing: the hourly check that emails Dan and Lee when no digest has been written for two hours (promised to IT, build by 9 Oct), and ISIT task monitoring on the server after week of 19 Oct. No metrics dashboard in ISIT tooling.</t>
         </is>
       </c>
       <c r="K22" s="21" t="inlineStr">
         <is>
-          <t>IT reply Q10; scan-state.json (since v2.45); WEEK-PLAN item 33. Owner: Dan (alert flow), ISIT (task monitoring). Date: 9 Oct and 18 Oct.</t>
+          <t>IT reply Q10; scan-state.json (since v2.45); WEEK-PLAN item 33. Owner: Dan (alert flow), ISIT (task monitoring). Date: 9 Oct and week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="K24" s="21" t="inlineStr">
         <is>
-          <t>Scan output 29 Sep (this pack, "Test summary"); rolling handoff entry 42.4 (sizes). Owner: Dan (projection), ISIT (server capacity). Date: 18 Oct.</t>
+          <t>Scan output 29 Sep (this pack, "Test summary"); rolling handoff entry 42.4 (sizes). Owner: Dan (projection), ISIT (server capacity). Date: week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="J25" s="19" t="inlineStr">
         <is>
-          <t>Not reviewed. The IT reply answered the ten security questions (accounts, no secrets, permissions, data location, the signed intake URL, the hashed password gates on the precharge, AAB and Help Centre pages, no external services). Planned as milestone M8b: submit for Architecture, Security and Governance review after the 18 Oct transfer, in November. v2, three findings the review must see, raised by the maintainers: the precharge gate is a curtain not a lock (page readable without the password; the requests folder reachable by URL; server-side IIS authentication needed before production, F-25); those request files carry employee names and work emails (F-70, closed by fixing F-25); the intake URL with its signature is a literal in both tool files, so anyone who can open a tool can post into the intake (KE-10, for ISIT to rate).</t>
+          <t>Not reviewed. The IT reply answered the ten security questions (accounts, no secrets, permissions, data location, the signed intake URL, the hashed password gates on the precharge, AAB and Help Centre pages, no external services). Planned as milestone M8b: submit for Architecture, Security and Governance review after the week of 19 Oct transfer, in November. v2, three findings the review must see, raised by the maintainers: the precharge gate is a curtain not a lock (page readable without the password; the requests folder reachable by URL; server-side IIS authentication needed before production, F-25); those request files carry employee names and work emails (F-70, closed by fixing F-25); the intake URL with its signature is a literal in both tool files, so anyone who can open a tool can post into the intake (KE-10, for ISIT to rate).</t>
         </is>
       </c>
       <c r="K25" s="21" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="J27" s="19" t="inlineStr">
         <is>
-          <t>Escalation today is to Technical Services, not the Service Desk: Dan Plant (script, dashboards, flows), Lee Arnold (co-owner), Adam Snyder (server, from 18 Oct), the tool maintainers per tool. A contact matrix is on the "Support Model (RACI)" sheet. Not yet loaded into the Service Desk.</t>
+          <t>Escalation today is to Technical Services, not the Service Desk: Dan Plant (script, dashboards, flows), Lee Arnold (co-owner), Adam Snyder (server, from week of 19 Oct), the tool maintainers per tool. A contact matrix is on the "Support Model (RACI)" sheet. Not yet loaded into the Service Desk.</t>
         </is>
       </c>
       <c r="K27" s="21" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="J28" s="19" t="inlineStr">
         <is>
-          <t>Every feature was proven on a test set and, for the flows, in test mode before it went live, and the proof is recorded per change in the handoff; the tools session hash-verifies each deployment. No consolidated test summary had been written; one is on the "Test summary" sheet. Warranty results come from the dual run (18 Oct to 6 Nov). v2: reporting-tools test records by revision (SSORT 144 to 153, WCGRRT 160 to 166), first-hand from SSORT 149 and WCGRRT 166, reconstructed from hashes before that, the gap stated; Precharge Pro suite (eleven harnesses, 47 physics scenarios, per-rig scope proof), records for Rev 83 to 87, two disclosures (Rev 86 encoding defect for 13 hours, no figure affected; the gate-check harness cannot currently run). Verification of the calculator is per rig: 4 of 13 rigs verified, 2 in progress, 7 not reviewed.</t>
+          <t>Every feature was proven on a test set and, for the flows, in test mode before it went live, and the proof is recorded per change in the handoff; the tools session hash-verifies each deployment. No consolidated test summary had been written; one is on the "Test summary" sheet. Warranty results come from the dual run (week of 19 Oct to 13 Nov). v2: reporting-tools test records by revision (SSORT 144 to 153, WCGRRT 160 to 166), first-hand from SSORT 149 and WCGRRT 166, reconstructed from hashes before that, the gap stated; Precharge Pro suite (eleven harnesses, 47 physics scenarios, per-rig scope proof), records for Rev 83 to 87, two disclosures (Rev 86 encoding defect for 13 hours, no figure affected; the gate-check harness cannot currently run). Verification of the calculator is per rig: 4 of 13 rigs verified, 2 in progress, 7 not reviewed.</t>
         </is>
       </c>
       <c r="K28" s="21" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="K37" s="21" t="inlineStr">
         <is>
-          <t>"DR and early-life support" sheet; SCANNER-SERVER-MIGRATION-IT-HANDOFF.md §6. Owner: Dan, then ISIT DR Lead. Date: 18 Oct.</t>
+          <t>"DR and early-life support" sheet; SCANNER-SERVER-MIGRATION-IT-HANDOFF.md §6. Owner: Dan, then ISIT DR Lead. Date: week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="J38" s="19" t="inlineStr">
         <is>
-          <t>Not tested formally. The dual run 18 Oct to 6 Nov is itself a live test of failover between the PC and the server. A rebuild-from-nothing test on the server (delete D:\TSC-Dashboard, rebuild from the repository, full rescan, compare counts) is proposed during the dual run.</t>
+          <t>Not tested formally. The dual run week of 19 Oct to 13 Nov is itself a live test of failover between the PC and the server. A rebuild-from-nothing test on the server (delete D:\TSC-Dashboard, rebuild from the repository, full rescan, compare counts) is proposed during the dual run.</t>
         </is>
       </c>
       <c r="K38" s="21" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>ISIT (Adam Snyder) from 18 Oct</t>
+          <t>ISIT (Adam Snyder) from week of 19 Oct</t>
         </is>
       </c>
       <c r="C3" s="19" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="F3" s="19" t="inlineStr">
         <is>
-          <t>Adam Snyder, ISIT. Until 18 Oct: Dan's PC, Dan.</t>
+          <t>Adam Snyder, ISIT. Until week of 19 Oct: Dan's PC, Dan.</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="C2" s="19" t="inlineStr">
         <is>
-          <t>Domain, service account (from 18 Oct)</t>
+          <t>Domain, service account (from week of 19 Oct)</t>
         </is>
       </c>
       <c r="D2" s="19" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="E2" s="19" t="inlineStr">
         <is>
-          <t>Serves http://sdrlazneuiis01d.corp.local:8080/sacred/... and /SSORT/. Scanner folder D:\TSC-Dashboard from 18 Oct.</t>
+          <t>Serves http://sdrlazneuiis01d.corp.local:8080/sacred/... and /SSORT/. Scanner folder D:\TSC-Dashboard from week of 19 Oct.</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3235,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Dan's PC today; server from 18 Oct (mechanism to decide, ORR item 8)</t>
+          <t>Dan's PC today; server from week of 19 Oct (mechanism to decide, ORR item 8)</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
@@ -5279,7 +5279,7 @@
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>18 Oct to 6 Nov 2026 (planned)</t>
+          <t>week of 19 Oct to 13 Nov 2026 (planned)</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
@@ -5617,7 +5617,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>18 Oct: transfer with Adam Snyder. 18 Oct to 6 Nov: dual run, Dan on call, daily count comparison. 6 Nov: Dan's PC task disabled; ISIT own the task; Dan owns the script. 6 Nov to Feb 2027: ISIT shadow-run, monthly note from Dan. Feb 2027: ISIT accept as a supported service (M11).</t>
+          <t>week of 19 Oct: transfer with Adam Snyder. week of 19 Oct to 13 Nov: dual run, Dan on call, daily count comparison. 6 Nov: Dan's PC task disabled; ISIT own the task; Dan owns the script. 6 Nov to Feb 2027: ISIT shadow-run, monthly note from Dan. Feb 2027: ISIT accept as a supported service (M11).</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5687,7 +5687,7 @@
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>Decide how the three report libraries reach the server under the service account (scheduled pull or sync); build it on 18 Oct</t>
+          <t>Decide how the three report libraries reach the server under the service account (scheduled pull or sync); build it on week of 19 Oct</t>
         </is>
       </c>
       <c r="C2" s="19" t="inlineStr">
@@ -5697,7 +5697,7 @@
       </c>
       <c r="D2" s="19" t="inlineStr">
         <is>
-          <t>10 Oct (decision), 18 Oct (build)</t>
+          <t>10 Oct (decision), week of 19 Oct (build)</t>
         </is>
       </c>
       <c r="E2" s="19" t="inlineStr">
@@ -5822,7 +5822,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>18 Oct; 6 Nov</t>
+          <t>week of 19 Oct; 6 Nov</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
@@ -5847,7 +5847,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>18 Oct</t>
+          <t>week of 19 Oct</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
@@ -5897,7 +5897,7 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>18 Oct</t>
+          <t>week of 19 Oct</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
@@ -5997,7 +5997,7 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>18 Oct</t>
+          <t>week of 19 Oct</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>18 Oct; 6 Nov</t>
+          <t>week of 19 Oct; 6 Nov</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -6328,6 +6328,33 @@
       <c r="E27" s="19" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>8 / 15</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>PRODUCTION HOME, not yet accounted for: the sacred server sdrlazneuiis01d is the sandbox. After the transfer the pages, the share and the scheduled task still run on it. ISIT to say whether it becomes the production server or a production server is built, and plan the cutover (URL change in the tools, the notification flows, the SSORT write-back share and the rigs' bookmarks). Until then nothing is in production, whatever the task runs under.</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>ISIT Infrastructure / Adam Snyder, with Dan</t>
+        </is>
+      </c>
+      <c r="D28" s="19" t="inlineStr">
+        <is>
+          <t>10 Oct (decision); build and cutover Nov to Jan, estimate</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>Open, critical path</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan item 40 and ORR open action: sending identity for the notification flows (shared mailbox now, service account at handover; no rebuild)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A2:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col width="2.5703125" customWidth="1" style="14" min="1" max="1"/>
@@ -5644,7 +5644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6358,6 +6358,33 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>2 / 17</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t>SENDING IDENTITY for the notification flows: today every notification email goes out under Dan's Office 365 connection. ISIT to create (a) a shared mailbox now, with Send As for Dan and Lee, so the From (Send as) field on the thirteen email cards can be set this month, and (b) the service account for the flows alongside the server account, so each flow's connections are swapped and the account added as owner at handover. No rebuild; no export/import (that would change the HTTP trigger URLs in the tools).</t>
+        </is>
+      </c>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>ISIT (Exchange, Power Platform admin) with Dan</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>10 Oct (shared mailbox); week of 19 Oct (service account)</t>
+        </is>
+      </c>
+      <c r="E29" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Meeting-notes and Viren emails as Word files with the one-page PDF; ORR v2 to REV 167/154 with KE-11 and KE-12; Audit-SurfaceTestRecords.ps1 for rolling handoff entry 45; entries 44 and 45 replied; Day 1 pack v4 and ORR return v2 filed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:K39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col width="2.5703125" customWidth="1" style="14" min="1" max="1"/>
@@ -2796,7 +2796,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT and SSORT reporting tools (REV 166, REV 153)</t>
+          <t>WCGRRT and SSORT reporting tools (REV 167, REV 154)</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>SSORT index.html (REV 153) and the COC dashboard copy.</t>
+          <t>SSORT index.html (REV 154) and the COC dashboard copy.</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT REV 166 (TSC Rig Reporting Tool)</t>
+          <t>WCGRRT REV 167 (TSC Rig Reporting Tool)</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 153 (Subsea Onboard Reporting Tool)</t>
+          <t>SSORT REV 154 (Subsea Onboard Reporting Tool)</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -3662,7 +3662,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 153 (verified live 30 Sep: 6,800,443 bytes, sha256 44cb4db89d2c…)</t>
+          <t>SSORT REV 154 (verified live 1 Oct: 6,804,809 bytes, sha256 f70d21f678b0…)</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -3689,7 +3689,7 @@
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT REV 166 (verified live 30 Sep: 3,340,404 bytes, sha256 83929b1a6749…)</t>
+          <t>WCGRRT REV 167 (verified live 1 Oct: 3,342,479 bytes, sha256 c916a062d457…)</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
@@ -3859,7 +3859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>The OEM copy's 30 MB refusal now counts the attached test records (from REV 153)</t>
+          <t>The OEM copy's 30 MB refusal now counts the attached test records (from REV 154)</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
@@ -4901,6 +4901,70 @@
       <c r="F33" s="19" t="inlineStr">
         <is>
           <t>ISIT with Dan; Lee (data owner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>RT KE-11</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>EHBS timer delay (B minus A) never computed while the form was filled in; posted empty on every EHBS test from either tool unless the crew saved, reloaded and restored</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Reported from a rig 30 Sep; ehbs_tim_delay empty in posted EHBS tests before 1 Oct</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>Recoverable: delay = shearStarts minus csrStops, both posted; the dashboard can derive it for display, labelled derived</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>CLOSED 1 Oct: WCGRRT 167 / SSORT 154 recompute on input. Posted-data audit by Dan (scanner side) to count affected reports</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>RT KE-12</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>HIGH, data loss: restoring a saved SSORT surface-test tile rendered the rig-keyed form as a placeholder and the next autosave overwrote the saved readings with nothing (five of seven forms rig-keyed; restore path listed four of seven types)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>A restored Acoustic, EHBS or Surface Drawdown record could lose its readings before posting; reach in posted reports unknown from the tool side</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>None before the fix; WCGRRT never had it</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>CLOSED 1 Oct: SSORT 154 shared renderer, tile keeps its own soak data, restore rebuilds after onAssetChange. Audit of posted reports (sbopData with testType set and an empty soak) by Dan</t>
+        </is>
+      </c>
+      <c r="F35" s="19" t="inlineStr">
+        <is>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -5375,7 +5439,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Pass; live file 44cb4db89d2c matches the REV 153 folder</t>
+          <t>Pass; live file f70d21f678b0 matches the REV 154 folder</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -5402,7 +5466,7 @@
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>Pass; live file 83929b1a6749 matches the folder</t>
+          <t>Pass; live file c916a062d457 matches the folder</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -5644,7 +5708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6385,6 +6449,60 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>11 / 19</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Audit posted reports for the SSORT restore defect (RT KE-12) and the empty EHBS timer delay (RT KE-11): count sbopData tiles with a testType and an empty soak, and EHBS tests with both times but no delay; name rig and date for any lost soak block so the crew's saved file can be recovered</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>Dan (scanner side, Audit-SurfaceTestRecords.ps1)</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>9 Oct</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>Retake Day 1 training screenshots 1 and 17 (revision badges) on WCGRRT 167 / SSORT 154; every other shot unaffected</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>Dan with the dashboard session, from the deployed files</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>12 Oct (packs final)</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
CoC tracker rebuilt: SACRED handoff on the SSCE loop it must keep, ORR rows, class module; Ronnie's API Std 53 session on workshop day 3 (agenda draft 2); class agenda draft 9; entries 46 and 47 replied
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A2:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col width="2.5703125" customWidth="1" style="14" min="1" max="1"/>
@@ -3028,7 +3028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3848,6 +3848,50 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>WCE Certificate of Conformance tracker, rebuilt (Seadrill_WCE_COC_Tracker.html, built 30 Sep 2026 on the Maximo flat export; handoff received 2 Oct)</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>One HTML file: data, logo and code embedded; opens from a share, SharePoint or an attachment; no server</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>Maximo extract (master record; refresh by Update from Excel + Save copy, or rebuild with build_tracker_v3.py); reference tables carried inside the file</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Manpreet Singh (owner, maintainer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>WCE COC Dashboard, REV6 era (Seadrill_WCE_COC_Dashboard.html on \\sdrlazneuiis01d\SSORT): the SSCE request front door and the scanner write-back target</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>SSORT share; APP_DATA block with the ssce folder</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>cocDashboardPath; SSCE-REQUESTS-INTEGRATION-CONTRACT.md</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Dan (scanner side); Manpreet (file). Superseded by the rebuilt tracker once the SSCE path is ported (COC-TRACKER-SACRED-HANDOFF.md)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3859,7 +3903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4965,6 +5009,166 @@
       <c r="F35" s="19" t="inlineStr">
         <is>
           <t>Dan Plant (owner); built with the reporting-tools session</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>COC KE-01</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>The rebuilt CoC tracker has no Request button and no APP_DATA block: the SSCE request path and the scanner's approved-request write-back do not work against it</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>If the rebuilt file replaces the REV6-era COC Dashboard on the SSORT share, no new SSCE request can be raised and the scanner logs "could not find the embedded APP_DATA block" every run</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Keep the REV6-era file on the share as the SSCE front door until the port is done</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>Port the Request path and available/assignedTo into the rebuilt tracker, then re-point the scanner write-back (COC-TRACKER-SACRED-HANDOFF.md option 1); decision by 10 Oct</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>Manpreet Singh with Dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>COC KE-02</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>1,969 of 3,364 fleet components (59%) carry no usable due date in the Maximo extract and cannot be scored; worst West Phoenix, West Elara and the Choke &amp; Kill manifold</t>
+        </is>
+      </c>
+      <c r="C37" s="19" t="inlineStr">
+        <is>
+          <t>Status tiers understate the expired and due populations</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>Shown as "No date on file", never guessed</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>Data entry in Maximo (issued and expiry dates); tracked by the rig and the CoC owner</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>Manpreet Singh; rig maintenance supervisors</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t>COC KE-03</t>
+        </is>
+      </c>
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>Shared Capital (0960) has no components in the Maximo extract; the 604 items are carried over from the v2 workbook inside the file</t>
+        </is>
+      </c>
+      <c r="C38" s="19" t="inlineStr">
+        <is>
+          <t>The spares register is a snapshot until Maximo exports it</t>
+        </is>
+      </c>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>Carry-over merged automatically; replaced the day Maximo exports them</t>
+        </is>
+      </c>
+      <c r="E38" s="19" t="inlineStr">
+        <is>
+          <t>Maximo export to include site 0960</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
+        <is>
+          <t>Manpreet Singh; Maximo admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>COC KE-04</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>Compliance ticks, remarks and Synergi numbers live in the viewer's own browser (localStorage), not in the file</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>Annotations do not travel with a copy, are not shared, and vanish when site data is cleared</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>By design; anything shared belongs in Maximo or Synergi</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>None planned; recorded as a design limit (ORR 27 retention also applies)</t>
+        </is>
+      </c>
+      <c r="F39" s="19" t="inlineStr">
+        <is>
+          <t>Manpreet Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>COC KE-05</t>
+        </is>
+      </c>
+      <c r="B40" s="19" t="inlineStr">
+        <is>
+          <t>Two Choke &amp; Kill SFIs (336.CK1.250, 336.CK1.270) have no category mapping; a genuinely new SFI falls back to the Maximo CATEGORY text and shows as Not defined; the auto-refresh link depends on the host allowing cross-origin download</t>
+        </is>
+      </c>
+      <c r="C40" s="19" t="inlineStr">
+        <is>
+          <t>Items grouped under the SFI group name; auto-refresh silently keeps embedded data</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
+        <is>
+          <t>Add to the v2 Category sheet and rebuild; use Update from Excel</t>
+        </is>
+      </c>
+      <c r="E40" s="19" t="inlineStr">
+        <is>
+          <t>Handoff §9 items 4, 7, 8</t>
+        </is>
+      </c>
+      <c r="F40" s="19" t="inlineStr">
+        <is>
+          <t>Manpreet Singh</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6503,6 +6707,33 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>19 / 22</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>CoC tracker return received as Manpreet's handoff (2 Oct): components, runbook, storage and known gaps filled from it. DECIDE the SSCE request path for the rebuilt tracker (port the Request button and available/assignedTo, keep both files, or move the form to SSORT) so the 20 Oct class teaches one file</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>Dan with Manpreet Singh and Lee</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>10 Oct</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Plan item 44: port the Request path back into the rebuilt CoC tracker and re-point the scanner write-back; ORR action updated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -6715,7 +6715,7 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>CoC tracker return received as Manpreet's handoff (2 Oct): components, runbook, storage and known gaps filled from it. DECIDE the SSCE request path for the rebuilt tracker (port the Request button and available/assignedTo, keep both files, or move the form to SSORT) so the 20 Oct class teaches one file</t>
+          <t>CoC tracker return received as Manpreet's handoff (2 Oct). DECIDED 2 Oct: the Request path and available/assignedTo are ported back into the rebuilt tracker from SACRED's build and the scanner write-back re-pointed (plan item 44); acceptance test before 10 Oct, live swap after; Manpreet carries the two fields through his refresh</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
@@ -6725,12 +6725,12 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>10 Oct</t>
+          <t>9 Oct (port, scanner v2.77); 10 Oct (acceptance); live swap after</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build freeze 12 Oct (entry 48) on the ORR and the pack plan; pack v6 and ORR return v3 filed; superintendents bring their own laptops
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:K39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col width="2.5703125" customWidth="1" style="14" min="1" max="1"/>
@@ -2796,7 +2796,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT and SSORT reporting tools (REV 167, REV 154)</t>
+          <t>WCGRRT and SSORT reporting tools (REV 167, REV 156)</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>SSORT index.html (REV 154) and the COC dashboard copy.</t>
+          <t>SSORT index.html (REV 156) and the COC dashboard copy.</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 154 (Subsea Onboard Reporting Tool)</t>
+          <t>SSORT REV 156 (Subsea Onboard Reporting Tool)</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -3662,7 +3662,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 154 (verified live 1 Oct: 6,804,809 bytes, sha256 f70d21f678b0…)</t>
+          <t>SSORT REV 156 (deployed 2 Oct: 6,893,201 bytes; hash to follow in the tools' test records; 154 verified 1 Oct f70d21f678b0…)</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>The OEM copy's 30 MB refusal now counts the attached test records (from REV 154)</t>
+          <t>The OEM copy's 30 MB refusal now counts the attached test records (from REV 156)</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
@@ -5643,7 +5643,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Pass; live file f70d21f678b0 matches the REV 154 folder</t>
+          <t>Pass; live file f70d21f678b0 matches the REV 156 folder</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -5912,7 +5912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6734,6 +6734,33 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>17 / 9</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t>BUILD FREEZE set by Dan 2 Oct: from 12 Oct to after the class on 20 Oct neither reporting tool changes unless a rig is losing work (data loss, a failed or silent post). Frozen builds are whatever is live on 12 Oct (today SSORT 156, WCGRRT 167). Held items logged in the rolling handoff and shipped in order after. Recorded in the tools' runbook §8 (ORR return v3)</t>
+        </is>
+      </c>
+      <c r="C33" s="19" t="inlineStr">
+        <is>
+          <t>Dan (rule); reporting-tools session (holds)</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>12 Oct to 20 Oct</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Day 2 scripts made definite: Ask SACRED AI on the trainer's laptop only; SSCE requests from the existing COC Dashboard, rebuilt tracker for status; CoC port (item 44) moves to after the class
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -5030,7 +5030,7 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Keep the REV6-era file on the share as the SSCE front door until the port is done</t>
+          <t>Keep the REV6-era file on the share as the SSCE front door until the port is done (through the class; port after 21 Oct)</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>9 Oct (port, scanner v2.77); 10 Oct (acceptance); live swap after</t>
+          <t>After the class (Dan, 3 Oct): port and scanner v2.77 from 21 Oct, acceptance, then live swap. The class raises requests from the existing COC Dashboard</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Day 2 scripts made definite: Ask SACRED AI on the trainer's laptop only; SSCE requests from the existing COC Dashboard, rebuilt tracker for status; CoC port (item 44) moves to after the class"
This reverts commit 38bb4814c318b4759da286847fdc961f0b7db67f.
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -5030,7 +5030,7 @@
       </c>
       <c r="D36" s="19" t="inlineStr">
         <is>
-          <t>Keep the REV6-era file on the share as the SSCE front door until the port is done (through the class; port after 21 Oct)</t>
+          <t>Keep the REV6-era file on the share as the SSCE front door until the port is done</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>After the class (Dan, 3 Oct): port and scanner v2.77 from 21 Oct, acceptance, then live swap. The class raises requests from the existing COC Dashboard</t>
+          <t>9 Oct (port, scanner v2.77); 10 Oct (acceptance); live swap after</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Entry 49 (SSORT 157): Auriga wrong-sheet count as a database query; ORR to SSORT 157 with KE-14; ORR return v4 filed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -2796,7 +2796,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT and SSORT reporting tools (REV 167, REV 156)</t>
+          <t>WCGRRT and SSORT reporting tools (REV 167, REV 157)</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>SSORT index.html (REV 156) and the COC dashboard copy.</t>
+          <t>SSORT index.html (REV 157) and the COC dashboard copy.</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 156 (Subsea Onboard Reporting Tool)</t>
+          <t>SSORT REV 157 (Subsea Onboard Reporting Tool)</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -3662,7 +3662,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 156 (deployed 2 Oct: 6,893,201 bytes; hash to follow in the tools' test records; 154 verified 1 Oct f70d21f678b0…)</t>
+          <t>SSORT REV 157 (verified live 5 Oct: 6,895,584 bytes, sha256 ba2ddd573e99…; 154 verified 1 Oct f70d21f678b0…)</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -3903,7 +3903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>The OEM copy's 30 MB refusal now counts the attached test records (from REV 156)</t>
+          <t>The OEM copy's 30 MB refusal now counts the attached test records (from REV 157)</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
@@ -5169,6 +5169,38 @@
       <c r="F40" s="19" t="inlineStr">
         <is>
           <t>Manpreet Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>RT KE-14</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="inlineStr">
+        <is>
+          <t>SSORT Daily Checks panel built once before the rig was picked and never rebuilt: West Auriga (and potentially West Saturn, Sevan Louisiana) recorded against Capella's sheet</t>
+        </is>
+      </c>
+      <c r="C41" s="19" t="inlineStr">
+        <is>
+          <t>Rounds recorded against the wrong rig's sheet; readings not wrong but taken on the wrong items list; the two sheets share no keys, so no reading lands on a wrong item</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>None before the fix</t>
+        </is>
+      </c>
+      <c r="E41" s="19" t="inlineStr">
+        <is>
+          <t>CLOSED 5 Oct: SSORT 157 rebuilds the panel on rig change, carrying readings across. Count of affected Auriga rounds from SACRED DATA (database/query-auriga-wrong-sheet.sql) to the tools session</t>
+        </is>
+      </c>
+      <c r="F41" s="19" t="inlineStr">
+        <is>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5675,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Pass; live file f70d21f678b0 matches the REV 156 folder</t>
+          <t>Pass; live file f70d21f678b0 matches the REV 157 folder</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Entry 49.4 answered from SACRED DATA: 2 Auriga and 1 Saturn rounds taken on Capella's sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A2:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
   <cols>
     <col width="2.5703125" customWidth="1" style="14" min="1" max="1"/>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>CLOSED 5 Oct: SSORT 157 rebuilds the panel on rig change, carrying readings across. Count of affected Auriga rounds from SACRED DATA (database/query-auriga-wrong-sheet.sql) to the tools session</t>
+          <t>CLOSED 5 Oct: SSORT 157 rebuilds the panel on rig change, carrying readings across. Reach counted from SACRED DATA on 5 Oct: West Auriga 2 of 72 rounds (28 Aug, 4 Oct), West Saturn 1 of 74 (18 Aug); taken back to the rigs by the tools session</t>
         </is>
       </c>
       <c r="F41" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Entry 51 filed and answered; frozen builds now WCGRRT 168 / SSORT 158
Tools session shipped SSORT 158 (CBM and surface-test names carry the
equipment or test type) and WCGRRT 168 (Save to File no longer posts).
Reply: agreed on no timestamp; asks them to check gate valves with the
serial blank and to state the slug rule for the recovery; Day 1 pack
still says SSORT 156. ORR workbook: 168/158, RT KE-15 and KE-16, test
row, three open actions. Day 2 docs and UAT form on 168/158/v2.79.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKpkuLyV6bHMBgkcjiDHio
</commit_message>
<xml_diff>
--- a/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
+++ b/Operation_Readiness_Review_ORR_Checklist_SACRED_v2.xlsx
@@ -2796,7 +2796,7 @@
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT and SSORT reporting tools (REV 167, REV 157)</t>
+          <t>WCGRRT and SSORT reporting tools (REV 168, REV 158)</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>SSORT index.html (REV 157) and the COC dashboard copy.</t>
+          <t>SSORT index.html (REV 158) and the COC dashboard copy.</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Scanner Update-Dashboard.ps1 v2.74 + config.json + state files</t>
+          <t>Scanner Update-Dashboard.ps1 v2.78 (v2.79 to install 9 Oct) + config.json + state files</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
@@ -3500,7 +3500,7 @@
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT REV 167 (TSC Rig Reporting Tool)</t>
+          <t>WCGRRT REV 168 (TSC Rig Reporting Tool)</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 157 (Subsea Onboard Reporting Tool)</t>
+          <t>SSORT REV 158 (Subsea Onboard Reporting Tool)</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -3662,7 +3662,7 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>SSORT REV 157 (verified live 5 Oct: 6,895,584 bytes, sha256 ba2ddd573e99…; 154 verified 1 Oct f70d21f678b0…)</t>
+          <t>SSORT REV 158 (verified live 6 Oct: 6,897,196 bytes, sha256 6c06a4712ebf…; 157 verified 5 Oct ba2ddd573e99…)</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -3689,7 +3689,7 @@
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>WCGRRT REV 167 (verified live 1 Oct: 3,342,479 bytes, sha256 c916a062d457…)</t>
+          <t>WCGRRT REV 168 (verified live 6 Oct: 3,342,821 bytes, sha256 a723b6df13b6…; 167 verified 1 Oct c916a062d457…)</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
@@ -3903,7 +3903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5204,6 +5204,70 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>RT KE-15</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>SSORT named a CBM post by rig and date only: two different inspections on one rig on one day shared a file name and SharePoint kept the second (surface BOP tests the same)</t>
+        </is>
+      </c>
+      <c r="C42" s="19" t="inlineStr">
+        <is>
+          <t>Earlier inspections vanished from the dashboard, digests, Ask SACRED AI and SACRED DATA; NOV still received each. West Capella: 13 CBMs to NOV since 30 Sep, 4 CBM files kept (found 6 Oct from SACRED DATA)</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>One CBM per rig per day, or all as tiles in one report (historical). Lost versions recoverable from PostedReports version history; Dan restoring</t>
+        </is>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>CLOSED 6 Oct: SSORT 158 names the post by equipment plus serial, surface tests by test type. Residual open: two instances of one class on one day with the serial blank (e.g. different gate valves, position held in the model field) may still share a name; raised with the tools session 6 Oct</t>
+        </is>
+      </c>
+      <c r="F42" s="19" t="inlineStr">
+        <is>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>RT KE-16</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>WCGRRT Save to File posted the report to the dashboard before opening Save As, with no rig, date or size guard and no confirm (since at least REV 155)</t>
+        </is>
+      </c>
+      <c r="C43" s="19" t="inlineStr">
+        <is>
+          <t>Unattributed posts (the Vendor Surveillance file of 3 Oct); unfinished reports posted unasked; a draft saved after the finished report replaced it under the same name</t>
+        </is>
+      </c>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
+          <t>None a crew would have known to apply</t>
+        </is>
+      </c>
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>CLOSED 6 Oct: WCGRRT 168 removes the post from Save to File; Post Report keeps its guards. Watch: a rig that reached the dashboard only through Save to File goes quiet until a crew presses Post Report</t>
+        </is>
+      </c>
+      <c r="F43" s="19" t="inlineStr">
+        <is>
+          <t>Dan Plant (owner); built with the reporting-tools session</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5215,7 +5279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5816,6 +5880,33 @@
       <c r="E22" s="19" t="inlineStr">
         <is>
           <t>ORR-RETURN-PRECHARGE-PRO.md §2.5 B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>6 Oct 2026 (SSORT 158, WCGRRT 168)</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>RT KE-15 and KE-16 fixes: CBM and surface-test names separate; a corrected re-post replaces; OEM then Post Report gives one file; Save to File posts nothing; Post Report still refuses a blank rig</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>Transport disabled; reproduced on the live 167 first; live files hash-verified against the revision folders</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Pass; live files 6c06a4712ebf (SSORT 158) and a723b6df13b6 (WCGRRT 168)</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="inlineStr">
+        <is>
+          <t>ORR-Reporting-Tools/02-Test-records-ORR-19.md; rolling handoff entry 51</t>
         </is>
       </c>
     </row>
@@ -5944,7 +6035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6720,7 +6811,7 @@
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>Retake Day 1 training screenshots 1 and 17 (revision badges) on WCGRRT 167 / SSORT 154; every other shot unaffected</t>
+          <t>Retake Day 1 training screenshots 1 and 17 (revision badges) on WCGRRT 168 / SSORT 158 (frozen builds from 6 Oct); every other shot unaffected</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
@@ -6790,6 +6881,87 @@
       <c r="E33" s="19" t="inlineStr">
         <is>
           <t>Set</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>11 / 19</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>Recover the West Capella CBM reports overwritten before SSORT 158 (RT KE-15) from PostedReports version history, named as SSORT 158 would name them; check each against its NOV copy</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Dan with the dashboard session</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>9 Oct</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>CBM name with the serial blank: two instances of one class on one day (the 6 Oct gate valves) may still collide under SSORT 158; tools session to confirm and, if so, carry the model position in the name (losing work, so a freeze exception)</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>Reporting-tools session with Dan</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>Before 12 Oct</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>After WCGRRT 168: watch for any rig that goes quiet (it may have been reaching the dashboard only through Save to File, RT KE-16); a phone call, not a fix</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="inlineStr">
+        <is>
+          <t>Dan (dashboard Status page by-rig table)</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>6 to 20 Oct</t>
+        </is>
+      </c>
+      <c r="E36" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>

</xml_diff>